<commit_message>
fix: stop losing table data and report the files written
</commit_message>
<xml_diff>
--- a/tests/Input/Test_sheets.xlsx
+++ b/tests/Input/Test_sheets.xlsx
@@ -1,8 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Progetti\IA\TextConverter\tests\Input\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
@@ -11,7 +16,7 @@
     <sheet name="Dates" sheetId="2" r:id="rId2"/>
     <sheet name="Secret" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -21,7 +26,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="A2" authorId="0">
+    <comment ref="A2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -40,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Item</t>
   </si>
@@ -110,11 +115,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-  </numFmts>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,18 +170,27 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -227,7 +238,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema di Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -269,7 +280,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -301,9 +312,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -335,6 +347,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -510,11 +523,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -527,11 +540,12 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" s="4"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -546,7 +560,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -561,7 +575,7 @@
         <v>11.25</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -576,7 +590,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -590,7 +604,7 @@
       </c>
       <c r="D5">
         <f>SUM(D2:D4)</f>
-        <v>20.5</v>
+        <v>23.75</v>
       </c>
     </row>
   </sheetData>
@@ -606,11 +620,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -621,7 +638,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>46325</v>
       </c>
@@ -632,9 +649,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
-        <v>46326.60416666666</v>
+        <v>46326.604166666657</v>
       </c>
       <c r="B3" t="b">
         <v>0</v>
@@ -650,11 +667,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>

</xml_diff>